<commit_message>
proprietati. indexatori. turnuri hanoi. Triunghiul lui Sierpinskki
</commit_message>
<xml_diff>
--- a/AlgoritmiSiStructuriDeDate2/Prezenta Algoritmi.xlsx
+++ b/AlgoritmiSiStructuriDeDate2/Prezenta Algoritmi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Geoinformatica_Promotia_2025_2028\AlgoritmiSiStructuriDeDate2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4BF88D-6371-4E1F-98DA-8E8BCAB9A798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D088DE6-11D5-45EE-8591-76F7D7C54AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -744,7 +744,9 @@
       <c r="D3" s="6">
         <v>2</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="6">
+        <v>2</v>
+      </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -758,7 +760,7 @@
       <c r="P3" s="7"/>
       <c r="Q3" s="8">
         <f t="shared" ref="Q3:Q22" si="0">SUM(C3:P3)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R3" s="7"/>
     </row>
@@ -767,10 +769,13 @@
         <v>25</v>
       </c>
       <c r="C4" s="9"/>
+      <c r="E4" s="3">
+        <v>2</v>
+      </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R4" s="10"/>
     </row>
@@ -831,10 +836,13 @@
       <c r="C9" s="9">
         <v>2</v>
       </c>
+      <c r="E9" s="3">
+        <v>2</v>
+      </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="8">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R9" s="10"/>
     </row>
@@ -848,10 +856,13 @@
       <c r="D10" s="3">
         <v>2</v>
       </c>
+      <c r="E10" s="3">
+        <v>2</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R10" s="10"/>
     </row>
@@ -875,10 +886,13 @@
         <v>24</v>
       </c>
       <c r="C12" s="9"/>
+      <c r="E12" s="3">
+        <v>2</v>
+      </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R12" s="10"/>
     </row>
@@ -892,10 +906,13 @@
       <c r="D13" s="3">
         <v>2</v>
       </c>
+      <c r="E13" s="3">
+        <v>2</v>
+      </c>
       <c r="P13" s="10"/>
       <c r="Q13" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R13" s="10"/>
     </row>
@@ -923,10 +940,13 @@
       <c r="D15" s="3">
         <v>2</v>
       </c>
+      <c r="E15" s="3">
+        <v>2</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R15" s="10"/>
     </row>
@@ -995,10 +1015,13 @@
       <c r="D20" s="3">
         <v>2</v>
       </c>
+      <c r="E20" s="3">
+        <v>2</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R20" s="10"/>
     </row>
@@ -1024,10 +1047,13 @@
       <c r="D22" s="3">
         <v>2</v>
       </c>
+      <c r="E22" s="3">
+        <v>2</v>
+      </c>
       <c r="P22" s="10"/>
       <c r="Q22" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R22" s="10"/>
     </row>

</xml_diff>

<commit_message>
abstractizare si closest points
</commit_message>
<xml_diff>
--- a/AlgoritmiSiStructuriDeDate2/Prezenta Algoritmi.xlsx
+++ b/AlgoritmiSiStructuriDeDate2/Prezenta Algoritmi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Geoinformatica_Promotia_2025_2028\AlgoritmiSiStructuriDeDate2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083D86D4-F759-4629-A5E6-AD4E45A0BCAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CDADA65-74DF-4D69-9561-FFCC05153129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -872,10 +872,13 @@
       <c r="G10" s="3">
         <v>2</v>
       </c>
+      <c r="I10" s="3">
+        <v>2</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R10" s="10"/>
     </row>
@@ -934,10 +937,13 @@
       <c r="G13" s="3">
         <v>2</v>
       </c>
+      <c r="I13" s="3">
+        <v>2</v>
+      </c>
       <c r="P13" s="10"/>
       <c r="Q13" s="8">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R13" s="10"/>
     </row>
@@ -1064,10 +1070,13 @@
       <c r="H20" s="3">
         <v>2</v>
       </c>
+      <c r="I20" s="3">
+        <v>2</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R20" s="10"/>
     </row>
@@ -1105,10 +1114,13 @@
       <c r="H22" s="3">
         <v>2</v>
       </c>
+      <c r="I22" s="3">
+        <v>2</v>
+      </c>
       <c r="P22" s="10"/>
       <c r="Q22" s="8">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R22" s="10"/>
     </row>

</xml_diff>

<commit_message>
namespace, interfete si map generator
</commit_message>
<xml_diff>
--- a/AlgoritmiSiStructuriDeDate2/Prezenta Algoritmi.xlsx
+++ b/AlgoritmiSiStructuriDeDate2/Prezenta Algoritmi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Geoinformatica_Promotia_2025_2028\AlgoritmiSiStructuriDeDate2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52BBA07D-CF88-4F03-9903-8C8045713B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA22079-543A-4F0D-97A6-E725D5AAA715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -883,10 +883,13 @@
       <c r="J10" s="3">
         <v>2</v>
       </c>
+      <c r="K10" s="3">
+        <v>2</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R10" s="10"/>
     </row>
@@ -1134,10 +1137,13 @@
       <c r="J22" s="3">
         <v>2</v>
       </c>
+      <c r="K22" s="3">
+        <v>2</v>
+      </c>
       <c r="P22" s="10"/>
       <c r="Q22" s="8">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="R22" s="10"/>
     </row>

</xml_diff>